<commit_message>
Release v0.4.1 with explicit title column names
</commit_message>
<xml_diff>
--- a/excel/MediaCatalog_template.xlsx
+++ b/excel/MediaCatalog_template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" r:id="Rbd620c7116a84de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" r:id="R0b3f9a0dea634aaf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -387,7 +387,7 @@
         <x:v>Blu-ray.com URL</x:v>
       </x:c>
       <x:c r="C1" s="10" t="str">
-        <x:v>Release Title</x:v>
+        <x:v>Blu-ray.com Title</x:v>
       </x:c>
       <x:c r="D1" s="10" t="str">
         <x:v>IMDb URL</x:v>
@@ -396,7 +396,7 @@
         <x:v>IMDb ID</x:v>
       </x:c>
       <x:c r="F1" s="10" t="str">
-        <x:v>Title</x:v>
+        <x:v>IMDb Title</x:v>
       </x:c>
       <x:c r="G1" s="10" t="str">
         <x:v>Year</x:v>
@@ -12450,7 +12450,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R864f67fa65ad4f6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bde955467c8412f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
MediaCatalog v0.4.1: explicit title column names
Makes Blu-ray.com Title and IMDb Title canonical across both templates, embedded and standalone macros, headers, installer identity, tests, and documentation while retaining legacy aliases.
</commit_message>
<xml_diff>
--- a/excel/MediaCatalog_template.xlsx
+++ b/excel/MediaCatalog_template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" r:id="Rbd620c7116a84de0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog" sheetId="1" r:id="R0b3f9a0dea634aaf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -387,7 +387,7 @@
         <x:v>Blu-ray.com URL</x:v>
       </x:c>
       <x:c r="C1" s="10" t="str">
-        <x:v>Release Title</x:v>
+        <x:v>Blu-ray.com Title</x:v>
       </x:c>
       <x:c r="D1" s="10" t="str">
         <x:v>IMDb URL</x:v>
@@ -396,7 +396,7 @@
         <x:v>IMDb ID</x:v>
       </x:c>
       <x:c r="F1" s="10" t="str">
-        <x:v>Title</x:v>
+        <x:v>IMDb Title</x:v>
       </x:c>
       <x:c r="G1" s="10" t="str">
         <x:v>Year</x:v>
@@ -12450,7 +12450,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R864f67fa65ad4f6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bde955467c8412f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete Windows 7 compatibility fixes
</commit_message>
<xml_diff>
--- a/excel/MediaCatalog_template.xlsx
+++ b/excel/MediaCatalog_template.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Michael\Documents\Media\MediaCatalog\excel\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{F1440415-073F-4899-8806-A0B08472CEED}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="60" yWindow="15" windowWidth="23970" windowHeight="17970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -16,7 +11,6 @@
     <sheet name="Catalog" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 

</xml_diff>